<commit_message>
feat: add all-in-one payroll calculator formulas
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Lista_Pagave_Sistemi_Genit.xlsx
+++ b/Lista_Pagave_Sistemi_Genit.xlsx
@@ -1,12 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <calcPr calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
   <sheets>
     <sheet name="Punonjësit" sheetId="1" r:id="rId1"/>
     <sheet name="Parametrat" sheetId="2" r:id="rId2"/>
     <sheet name="Lista e Pagave" sheetId="3" r:id="rId3"/>
     <sheet name="Udhëzime" sheetId="4" r:id="rId4"/>
     <sheet name="Orari 31 Ditë" sheetId="5" r:id="rId5"/>
+    <sheet name="Kalkulatori" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -27484,4 +27486,191 @@
   </sheetData>
   <pageMargins left="0.3" right="0.3" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B21"/>
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KALKULATORI I PAGËS — ALL IN ONE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Të dhënat hyrëse</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>Vlera</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Paga bazë bruto</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Shtesa</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Orë shtesë</t>
+        </is>
+      </c>
+      <c r="B6" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Çmimi/orë shtesë</t>
+        </is>
+      </c>
+      <c r="B7" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Shpërblim</t>
+        </is>
+      </c>
+      <c r="B8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Paga bruto</t>
+        </is>
+      </c>
+      <c r="B10" s="3">
+        <f>=B4+B5+B6*B7+B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SS punonjës</t>
+        </is>
+      </c>
+      <c r="B11" s="3">
+        <f>=MIN(B10,Parametrat!$B$6)*Parametrat!$B$2/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SH punonjës</t>
+        </is>
+      </c>
+      <c r="B12" s="3">
+        <f>=B10*Parametrat!$B$3/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Paga e tatueshme</t>
+        </is>
+      </c>
+      <c r="B13" s="3">
+        <f>=MAX(0,B10-B11-B12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>TAP</t>
+        </is>
+      </c>
+      <c r="B14" s="3">
+        <f>=IF(B13&lt;=Parametrat!$B$7,0,IF(B13&lt;=Parametrat!$B$8,(B13-Parametrat!$B$7)*Parametrat!$B$9/100,(Parametrat!$B$8-Parametrat!$B$7)*Parametrat!$B$9/100+(B13-Parametrat!$B$8)*Parametrat!$B$10/100))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Paga neto</t>
+        </is>
+      </c>
+      <c r="B15" s="3">
+        <f>=B10-B11-B12-B14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SS punëdhënës</t>
+        </is>
+      </c>
+      <c r="B16" s="3">
+        <f>=MIN(B10,Parametrat!$B$6)*Parametrat!$B$4/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SH punëdhënës</t>
+        </is>
+      </c>
+      <c r="B17" s="3">
+        <f>=B10*Parametrat!$B$5/100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>Kosto totale punëdhënësi</t>
+        </is>
+      </c>
+      <c r="B18" s="3">
+        <f>=B10+B16+B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Shënim: ndrysho normat te Parametrat. Përdor Kalkulatorin për të kontrolluar bruto-në-neto para transferimit në listë.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>